<commit_message>
Auto stash before merge of "main" and "origin/main"
</commit_message>
<xml_diff>
--- a/Reporte_Tareas_2026-02-20.xlsx
+++ b/Reporte_Tareas_2026-02-20.xlsx
@@ -454,16 +454,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
     <col width="52" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1165,6 +1165,776 @@
       <c r="G20" s="2" t="inlineStr">
         <is>
           <t>clonacion</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>MODELO EOI</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>GUIAS EOI id=3</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Licitaciones</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>licitaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>MODELO EOI</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>GUIAS EOI id=14</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Licitaciones</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>licitaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>MODELO EOI</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>GUIAS EOI id=5</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Licitaciones</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>licitaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>MODELO EOI</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>GUIAS EOI id=4</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Licitaciones</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>licitaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>MEC</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Luis Jiménez Contreras</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>RRHH</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>rrhh</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>EJECUCIÓN EOI</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>GUIAS EOI id=20</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Licitaciones</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>licitaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>EJECUCIÓN EOI</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>GUIAS EOI id=6</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Licitaciones</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>licitaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>EJECUCIÓN EOI</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>GUIAS EOI id=7</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Licitaciones</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>licitaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>EJECUCIÓN EOI</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>GUIAS EOI id=8</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Licitaciones</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>licitaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>EJECUCIÓN EOI</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>GUIAS EOI id=10</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Licitaciones</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>licitaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>EJECUCIÓN EOI</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>GUIAS EOI id=11</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Licitaciones</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>licitaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>EJECUCIÓN EOI</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>GUIAS EOI id=12</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Licitaciones</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>licitaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>EJECUCIÓN EOI</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>GUIAS EOI id=13</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Licitaciones</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>licitaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>EJECUCIÓN EOI</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>GUIAS EOI id=15</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Licitaciones</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>licitaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>EJECUCIÓN EOI</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>GUIAS EOI id=17</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Licitaciones</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>licitaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>EJECUCIÓN EOI</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>GUIAS EOI id=23</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Licitaciones</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>licitaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>EJECUCIÓN EOI</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>GUIAS EOI id=16</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>Licitaciones</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>licitaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>EJECUCIÓN EOI</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>GUIAS EOI id=19</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Licitaciones</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>licitaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>EJECUCIÓN EOI</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>GUIAS EOI id=18</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>Licitaciones</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="F39" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>licitaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>EJECUCIÓN EOI</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>GUIAS EOI id=20</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>Licitaciones</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>licitaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>MF1005_3 Emma</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>MEC = 5795 // MEC = 5885</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>VAL 25</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="F41" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>clonacion</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>MEC</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Federico José Pérez Galindo</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>RRHH</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-26</t>
+        </is>
+      </c>
+      <c r="F42" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>rrhh</t>
         </is>
       </c>
     </row>
@@ -1179,16 +1949,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
     <col width="43" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1438,6 +2208,706 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>MODELO EOI</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>GUIAS EOI id=3</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Licitaciones</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>licitaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>MODELO EOI</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>GUIAS EOI id=14</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Licitaciones</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>licitaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>MODELO EOI</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>GUIAS EOI id=5</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Licitaciones</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>licitaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>MODELO EOI</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>GUIAS EOI id=4</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Licitaciones</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>licitaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>EJECUCIÓN EOI</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>GUIAS EOI id=20</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Licitaciones</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>licitaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>EJECUCIÓN EOI</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>GUIAS EOI id=6</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Licitaciones</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>licitaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>EJECUCIÓN EOI</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>GUIAS EOI id=7</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Licitaciones</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>licitaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>EJECUCIÓN EOI</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>GUIAS EOI id=8</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Licitaciones</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>licitaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>EJECUCIÓN EOI</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>GUIAS EOI id=10</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Licitaciones</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>licitaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>EJECUCIÓN EOI</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>GUIAS EOI id=11</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Licitaciones</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>licitaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>EJECUCIÓN EOI</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>GUIAS EOI id=12</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Licitaciones</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>licitaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>EJECUCIÓN EOI</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>GUIAS EOI id=13</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Licitaciones</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>licitaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>EJECUCIÓN EOI</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>GUIAS EOI id=15</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Licitaciones</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>licitaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>EJECUCIÓN EOI</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>GUIAS EOI id=17</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Licitaciones</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>licitaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>EJECUCIÓN EOI</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>GUIAS EOI id=23</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Licitaciones</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>licitaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>EJECUCIÓN EOI</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>GUIAS EOI id=16</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Licitaciones</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>licitaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>EJECUCIÓN EOI</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>GUIAS EOI id=19</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Licitaciones</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>licitaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>EJECUCIÓN EOI</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>GUIAS EOI id=18</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Licitaciones</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>licitaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>EJECUCIÓN EOI</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>GUIAS EOI id=20</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Licitaciones</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>licitaciones</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>MF1005_3 Emma</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>MEC = 5795 // MEC = 5885</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>VAL 25</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>Completada</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>clonacion</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>